<commit_message>
feat: 并入 LingXu Character OS v0.1（5 角色 + face_registry + visual rules）
- 01_CHARACTERS/{星澜,烬离,北寒溟,墨千,疏岚}：复制 _TEMPLATE 并填 character.md / face_dna.md / identity_anchor.md
- 04_DATABASE/face_index.csv|xlsx 换成 5 个真实角色；新增 face_registry.json（v0.1 原文件）
- 00_PROJECT_RULES/visual_style.md 补 v0.1 口径（PBR+SSS、禁网红脸、Face DNA 区分）
- 防撞脸互查：5 人两两相似度 <55%，无撞脸
- 01_CHARACTERS/README.md 迁移待办、character_compare.md 备注更新

来源：LingXu_Character_OS_v0.1.zip（用户提供）
</commit_message>
<xml_diff>
--- a/04_DATABASE/face_index.xlsx
+++ b/04_DATABASE/face_index.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +31,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +46,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,12 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,116 +440,116 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>角色</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>拼音ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>性别</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>年龄</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>阵营</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>属性</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>脸型</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>三庭</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>眉形</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>眼型</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>眼距</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>鼻型</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>下颌</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>唇型</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>个性标志</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Face DNA版本</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -576,7 +588,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>方鹅蛋65%+倒梯形35%</t>
+          <t>方鹅蛋 65% + 倒梯形 35%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -591,7 +603,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>成熟长杏眼/眼尾微挑</t>
+          <t>成熟冷感长杏眼（眼尾轻微上挑）</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -601,7 +613,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>中高鼻根+中直鼻梁+自然鼻头</t>
+          <t>中高鼻根 + 中直鼻梁 + 自然鼻头</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -611,7 +623,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>中等嘴宽/上薄下厚</t>
+          <t>中等嘴宽 / 上薄下厚</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -631,99 +643,375 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>示例数据，按 face_dna.md 校准</t>
+          <t>来自 v0.1 face_registry（identity_mark：保留已有身份图锁定）</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>烬离</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>jinli</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>镇墟司</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>成熟男性骨相脸</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>锐利但克制</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>明显下颌线</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>（待补）</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>来自 v0.1 face_registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>北寒溟</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>beihanming</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>男</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>镇墟司</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>水</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>长方脸</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>狭长眼</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>长方脸（独立水系冷感骨相）</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>狭长眼（冷色瞳）</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>骨感鼻梁</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>宽下颌</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>鼻梁旧伤</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>v001</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>示例数据，按 face_dna.md 校准</t>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>来自 v0.1 face_registry（合并原 spec：长方脸/狭长眼/骨感鼻梁/宽下颌/鼻梁旧伤）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>墨千</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>moqian</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>硬朗长方脸</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>深眼窝沉稳眼</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>厚重下颌</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>（待补）</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>来自 v0.1 face_registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>疏岚</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>shulan</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>重新锁定独立脸型（待定稿）</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>攻击性眼型</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>（待补）</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>（待补）</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>v001</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>来自 v0.1 face_registry（face_shape：重新锁定独立脸型）</t>
         </is>
       </c>
     </row>
@@ -838,7 +1126,6 @@
           <t>眉形</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>G 组</t>

</xml_diff>